<commit_message>
add listings, neighbourhoods, reviews staging models
</commit_message>
<xml_diff>
--- a/docs/airbnb-sttm.xlsx
+++ b/docs/airbnb-sttm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\dbt-projects\dbt-airbnb-project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F96CE0-C02A-48DA-9334-7E2F27A5217A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB630E9B-B4F7-4288-812F-278F80456125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="141">
   <si>
     <t>Destination Table</t>
   </si>
@@ -454,6 +454,15 @@
   </si>
   <si>
     <t>snapshot_date_id</t>
+  </si>
+  <si>
+    <t>Rename column, trim whitespaces</t>
+  </si>
+  <si>
+    <t>review_scores_cleanliness</t>
+  </si>
+  <si>
+    <t>review_scores_location</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1123,7 @@
         <v>16</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>87</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1144,7 +1153,7 @@
         <v>17</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -1964,7 +1973,7 @@
         <v>88</v>
       </c>
       <c r="B34" t="s">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="D34" t="s">
         <v>45</v>
@@ -1993,7 +2002,7 @@
         <v>88</v>
       </c>
       <c r="B35" t="s">
-        <v>106</v>
+        <v>140</v>
       </c>
       <c r="D35" t="s">
         <v>45</v>
@@ -2222,6 +2231,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add all rating related columns to stg_listings and downstream
</commit_message>
<xml_diff>
--- a/docs/airbnb-sttm.xlsx
+++ b/docs/airbnb-sttm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git-repos\dbt-projects\dbt-airbnb-project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C80122-D256-4B0D-AEBA-B035B5C4D117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F068952-ECBA-4AEC-8EC1-7F49C38EEEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{BBF274AC-B2B2-491E-9DB3-2437D80DB6CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw to Staging" sheetId="4" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="150">
   <si>
     <t>Destination Table</t>
   </si>
@@ -516,6 +516,18 @@
   </si>
   <si>
     <t>scd_property__listings</t>
+  </si>
+  <si>
+    <t>review_scores_checkin</t>
+  </si>
+  <si>
+    <t>review_score_communication</t>
+  </si>
+  <si>
+    <t>review_score_rating</t>
+  </si>
+  <si>
+    <t>review_score_checkin</t>
   </si>
 </sst>
 </file>
@@ -1107,11 +1119,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5ED6477-E8E4-4322-A2B1-C7E8A834095A}">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.26953125" customWidth="1"/>
     <col min="3" max="3" width="5.08984375" customWidth="1"/>
     <col min="4" max="4" width="26.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.36328125" bestFit="1" customWidth="1"/>
@@ -2089,7 +2101,7 @@
         <v>86</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="D36" t="s">
         <v>45</v>
@@ -2101,7 +2113,7 @@
         <v>81</v>
       </c>
       <c r="G36" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="H36" t="s">
         <v>45</v>
@@ -2113,62 +2125,62 @@
         <v>46</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
-      <c r="A40" t="s">
-        <v>111</v>
-      </c>
-      <c r="B40" t="s">
-        <v>119</v>
-      </c>
-      <c r="D40" t="s">
-        <v>45</v>
-      </c>
-      <c r="E40" t="s">
-        <v>16</v>
-      </c>
-      <c r="F40" t="s">
-        <v>112</v>
-      </c>
-      <c r="G40" t="s">
-        <v>72</v>
-      </c>
-      <c r="H40" t="s">
-        <v>45</v>
-      </c>
-      <c r="I40" t="s">
-        <v>16</v>
-      </c>
-      <c r="J40" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10">
-      <c r="A41" t="s">
-        <v>111</v>
-      </c>
-      <c r="B41" t="s">
-        <v>65</v>
-      </c>
-      <c r="D41" t="s">
-        <v>45</v>
-      </c>
-      <c r="E41" t="s">
-        <v>16</v>
-      </c>
-      <c r="F41" t="s">
-        <v>112</v>
-      </c>
-      <c r="G41" t="s">
-        <v>37</v>
-      </c>
-      <c r="H41" t="s">
-        <v>45</v>
-      </c>
-      <c r="I41" t="s">
-        <v>16</v>
-      </c>
-      <c r="J41" t="s">
-        <v>87</v>
+    <row r="37" spans="1:10">
+      <c r="A37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" t="s">
+        <v>147</v>
+      </c>
+      <c r="D37" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G37" t="s">
+        <v>147</v>
+      </c>
+      <c r="H37" t="s">
+        <v>45</v>
+      </c>
+      <c r="I37" t="s">
+        <v>17</v>
+      </c>
+      <c r="J37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
+      <c r="A38" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" t="s">
+        <v>81</v>
+      </c>
+      <c r="G38" t="s">
+        <v>105</v>
+      </c>
+      <c r="H38" t="s">
+        <v>45</v>
+      </c>
+      <c r="I38" t="s">
+        <v>17</v>
+      </c>
+      <c r="J38" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -2176,10 +2188,10 @@
         <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D42" t="s">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E42" t="s">
         <v>16</v>
@@ -2188,10 +2200,10 @@
         <v>112</v>
       </c>
       <c r="G42" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="H42" t="s">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="I42" t="s">
         <v>16</v>
@@ -2205,7 +2217,7 @@
         <v>111</v>
       </c>
       <c r="B43" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="D43" t="s">
         <v>45</v>
@@ -2217,7 +2229,7 @@
         <v>112</v>
       </c>
       <c r="G43" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H43" t="s">
         <v>45</v>
@@ -2234,10 +2246,10 @@
         <v>111</v>
       </c>
       <c r="B44" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="D44" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="E44" t="s">
         <v>16</v>
@@ -2246,16 +2258,16 @@
         <v>112</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
+        <v>106</v>
       </c>
       <c r="H44" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="I44" t="s">
         <v>16</v>
       </c>
       <c r="J44" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -2263,10 +2275,10 @@
         <v>111</v>
       </c>
       <c r="B45" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E45" t="s">
         <v>16</v>
@@ -2275,15 +2287,73 @@
         <v>112</v>
       </c>
       <c r="G45" t="s">
+        <v>10</v>
+      </c>
+      <c r="H45" t="s">
+        <v>45</v>
+      </c>
+      <c r="I45" t="s">
+        <v>16</v>
+      </c>
+      <c r="J45" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10">
+      <c r="A46" t="s">
+        <v>111</v>
+      </c>
+      <c r="B46" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" t="s">
+        <v>20</v>
+      </c>
+      <c r="E46" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>112</v>
+      </c>
+      <c r="G46" t="s">
+        <v>12</v>
+      </c>
+      <c r="H46" t="s">
+        <v>20</v>
+      </c>
+      <c r="I46" t="s">
+        <v>16</v>
+      </c>
+      <c r="J46" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" t="s">
         <v>66</v>
       </c>
-      <c r="H45" t="s">
-        <v>20</v>
-      </c>
-      <c r="I45" t="s">
-        <v>16</v>
-      </c>
-      <c r="J45" t="s">
+      <c r="D47" t="s">
+        <v>20</v>
+      </c>
+      <c r="E47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>112</v>
+      </c>
+      <c r="G47" t="s">
+        <v>66</v>
+      </c>
+      <c r="H47" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" t="s">
+        <v>16</v>
+      </c>
+      <c r="J47" t="s">
         <v>113</v>
       </c>
     </row>
@@ -2295,11 +2365,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1FA96D-39B5-4C35-B630-6E03D89B8F47}">
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.1796875" customWidth="1"/>
     <col min="4" max="4" width="29.90625" customWidth="1"/>
     <col min="5" max="5" width="27.6328125" customWidth="1"/>
@@ -2843,25 +2913,25 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
         <v>45</v>
       </c>
       <c r="E20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>44</v>
+        <v>145</v>
       </c>
       <c r="G20" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="H20" t="s">
         <v>45</v>
       </c>
       <c r="I20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>46</v>
@@ -2872,25 +2942,25 @@
         <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>148</v>
       </c>
       <c r="D21" t="s">
         <v>45</v>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>44</v>
+        <v>145</v>
       </c>
       <c r="G21" t="s">
-        <v>34</v>
+        <v>148</v>
       </c>
       <c r="H21" t="s">
         <v>45</v>
       </c>
       <c r="I21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>46</v>
@@ -2901,28 +2971,28 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F22" t="s">
         <v>145</v>
       </c>
       <c r="G22" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="H22" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2930,10 +3000,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="E23" t="s">
         <v>17</v>
@@ -2942,16 +3012,16 @@
         <v>145</v>
       </c>
       <c r="G23" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="H23" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I23" t="s">
         <v>17</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2959,28 +3029,28 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D24" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F24" t="s">
         <v>145</v>
       </c>
       <c r="G24" t="s">
-        <v>22</v>
+        <v>147</v>
       </c>
       <c r="H24" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="I24" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>144</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2988,233 +3058,233 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="D25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" t="s">
+        <v>33</v>
+      </c>
+      <c r="H25" t="s">
+        <v>45</v>
+      </c>
+      <c r="I25" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>44</v>
+      </c>
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" t="s">
+        <v>45</v>
+      </c>
+      <c r="I26" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" t="s">
         <v>21</v>
       </c>
-      <c r="E25" t="s">
-        <v>16</v>
-      </c>
-      <c r="F25" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" t="s">
-        <v>22</v>
-      </c>
-      <c r="H25" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
-      <c r="A26" s="6" t="s">
+      <c r="E27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>145</v>
+      </c>
+      <c r="G27" t="s">
+        <v>142</v>
+      </c>
+      <c r="H27" t="s">
+        <v>21</v>
+      </c>
+      <c r="I27" t="s">
+        <v>16</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7" t="s">
+      <c r="B28" t="s">
+        <v>139</v>
+      </c>
+      <c r="D28" t="s">
         <v>21</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>19</v>
+      <c r="E28" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" t="s">
+        <v>145</v>
+      </c>
+      <c r="G28" t="s">
+        <v>143</v>
+      </c>
+      <c r="H28" t="s">
+        <v>21</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:10">
-      <c r="A29" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>36</v>
+      <c r="A29" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" t="s">
+        <v>140</v>
+      </c>
+      <c r="D29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" t="s">
+        <v>145</v>
+      </c>
+      <c r="G29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B30" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G30" t="s">
-        <v>50</v>
-      </c>
-      <c r="H30" t="s">
-        <v>45</v>
-      </c>
-      <c r="I30" t="s">
-        <v>16</v>
-      </c>
-      <c r="J30" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
-      <c r="A31" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B31" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" t="s">
-        <v>44</v>
-      </c>
-      <c r="G31" t="s">
-        <v>51</v>
-      </c>
-      <c r="H31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" t="s">
-        <v>80</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10">
-      <c r="A32" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" t="s">
-        <v>132</v>
-      </c>
-      <c r="D32" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" t="s">
-        <v>44</v>
-      </c>
-      <c r="G32" t="s">
-        <v>52</v>
-      </c>
-      <c r="H32" t="s">
-        <v>21</v>
-      </c>
-      <c r="I32" t="s">
-        <v>17</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10">
-      <c r="A33" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" t="s">
-        <v>53</v>
-      </c>
-      <c r="D33" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" t="s">
-        <v>17</v>
-      </c>
-      <c r="F33" t="s">
-        <v>44</v>
-      </c>
-      <c r="G33" t="s">
-        <v>53</v>
-      </c>
-      <c r="H33" t="s">
-        <v>20</v>
-      </c>
-      <c r="I33" t="s">
-        <v>17</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10">
-      <c r="A34" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D34" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" t="s">
-        <v>44</v>
-      </c>
-      <c r="G34" t="s">
-        <v>54</v>
-      </c>
-      <c r="H34" t="s">
-        <v>45</v>
-      </c>
-      <c r="I34" t="s">
-        <v>17</v>
-      </c>
-      <c r="J34" s="5" t="s">
-        <v>46</v>
+      <c r="B34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -3222,25 +3292,25 @@
         <v>47</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D35" t="s">
         <v>45</v>
       </c>
       <c r="E35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F35" t="s">
         <v>44</v>
       </c>
       <c r="G35" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H35" t="s">
         <v>45</v>
       </c>
       <c r="I35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>46</v>
@@ -3251,25 +3321,25 @@
         <v>47</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D36" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="F36" t="s">
         <v>44</v>
       </c>
       <c r="G36" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H36" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="I36" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>46</v>
@@ -3280,10 +3350,10 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="D37" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E37" t="s">
         <v>17</v>
@@ -3292,16 +3362,16 @@
         <v>44</v>
       </c>
       <c r="G37" t="s">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="H37" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="I37" t="s">
         <v>17</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>46</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -3309,10 +3379,10 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D38" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E38" t="s">
         <v>17</v>
@@ -3321,7 +3391,7 @@
         <v>44</v>
       </c>
       <c r="G38" t="s">
-        <v>94</v>
+        <v>53</v>
       </c>
       <c r="H38" t="s">
         <v>20</v>
@@ -3330,7 +3400,7 @@
         <v>17</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>114</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -3338,10 +3408,10 @@
         <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D39" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E39" t="s">
         <v>17</v>
@@ -3350,16 +3420,16 @@
         <v>44</v>
       </c>
       <c r="G39" t="s">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="H39" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I39" t="s">
         <v>17</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -3367,10 +3437,10 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D40" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E40" t="s">
         <v>17</v>
@@ -3379,16 +3449,16 @@
         <v>44</v>
       </c>
       <c r="G40" t="s">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="H40" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I40" t="s">
         <v>17</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>116</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -3396,28 +3466,28 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>138</v>
+        <v>56</v>
       </c>
       <c r="D41" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E41" t="s">
         <v>16</v>
       </c>
       <c r="F41" t="s">
-        <v>141</v>
+        <v>44</v>
       </c>
       <c r="G41" t="s">
-        <v>142</v>
+        <v>56</v>
       </c>
       <c r="H41" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="I41" t="s">
         <v>16</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -3425,28 +3495,28 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>95</v>
       </c>
       <c r="D42" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E42" t="s">
         <v>17</v>
       </c>
       <c r="F42" t="s">
-        <v>141</v>
+        <v>44</v>
       </c>
       <c r="G42" t="s">
-        <v>143</v>
+        <v>95</v>
       </c>
       <c r="H42" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="I42" t="s">
         <v>17</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -3454,28 +3524,28 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>57</v>
       </c>
       <c r="D43" t="s">
         <v>35</v>
       </c>
       <c r="E43" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F43" t="s">
-        <v>141</v>
+        <v>44</v>
       </c>
       <c r="G43" t="s">
-        <v>22</v>
+        <v>94</v>
       </c>
       <c r="H43" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I43" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3483,243 +3553,270 @@
         <v>47</v>
       </c>
       <c r="B44" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="D44" t="s">
+        <v>35</v>
+      </c>
+      <c r="E44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" t="s">
+        <v>44</v>
+      </c>
+      <c r="G44" t="s">
+        <v>94</v>
+      </c>
+      <c r="H44" t="s">
+        <v>20</v>
+      </c>
+      <c r="I44" t="s">
+        <v>17</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10">
+      <c r="A45" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" t="s">
+        <v>35</v>
+      </c>
+      <c r="E45" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" t="s">
+        <v>44</v>
+      </c>
+      <c r="G45" t="s">
+        <v>94</v>
+      </c>
+      <c r="H45" t="s">
+        <v>20</v>
+      </c>
+      <c r="I45" t="s">
+        <v>17</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10">
+      <c r="A46" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" t="s">
+        <v>138</v>
+      </c>
+      <c r="D46" t="s">
         <v>21</v>
       </c>
-      <c r="E44" t="s">
-        <v>16</v>
-      </c>
-      <c r="F44" t="s">
-        <v>22</v>
-      </c>
-      <c r="G44" t="s">
-        <v>22</v>
-      </c>
-      <c r="H44" t="s">
-        <v>22</v>
-      </c>
-      <c r="I44" t="s">
-        <v>22</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10">
-      <c r="A45" s="6" t="s">
+      <c r="E46" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>141</v>
+      </c>
+      <c r="G46" t="s">
+        <v>142</v>
+      </c>
+      <c r="H46" t="s">
+        <v>21</v>
+      </c>
+      <c r="I46" t="s">
+        <v>16</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7" t="s">
+      <c r="B47" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" t="s">
         <v>21</v>
       </c>
-      <c r="E45" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J45" s="8" t="s">
-        <v>19</v>
+      <c r="E47" t="s">
+        <v>17</v>
+      </c>
+      <c r="F47" t="s">
+        <v>141</v>
+      </c>
+      <c r="G47" t="s">
+        <v>143</v>
+      </c>
+      <c r="H47" t="s">
+        <v>21</v>
+      </c>
+      <c r="I47" t="s">
+        <v>17</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:10">
-      <c r="A48" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>36</v>
+      <c r="A48" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>140</v>
+      </c>
+      <c r="D48" t="s">
+        <v>35</v>
+      </c>
+      <c r="E48" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" t="s">
+        <v>141</v>
+      </c>
+      <c r="G48" t="s">
+        <v>22</v>
+      </c>
+      <c r="H48" t="s">
+        <v>22</v>
+      </c>
+      <c r="I48" t="s">
+        <v>22</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>21</v>
+      </c>
+      <c r="E49" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" t="s">
+        <v>22</v>
+      </c>
+      <c r="G49" t="s">
+        <v>22</v>
+      </c>
+      <c r="H49" t="s">
+        <v>22</v>
+      </c>
+      <c r="I49" t="s">
+        <v>22</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I50" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J50" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
+      <c r="A53" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B53" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
+      <c r="A54" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" t="s">
         <v>61</v>
       </c>
-      <c r="D49" t="s">
-        <v>20</v>
-      </c>
-      <c r="E49" t="s">
-        <v>16</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="D54" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" t="s">
         <v>44</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G54" t="s">
         <v>100</v>
       </c>
-      <c r="H49" t="s">
-        <v>20</v>
-      </c>
-      <c r="I49" t="s">
-        <v>16</v>
-      </c>
-      <c r="J49" s="5" t="s">
+      <c r="H54" t="s">
+        <v>20</v>
+      </c>
+      <c r="I54" t="s">
+        <v>16</v>
+      </c>
+      <c r="J54" s="5" t="s">
         <v>117</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10">
-      <c r="A50" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B50" t="s">
-        <v>62</v>
-      </c>
-      <c r="D50" t="s">
-        <v>20</v>
-      </c>
-      <c r="E50" t="s">
-        <v>16</v>
-      </c>
-      <c r="F50" t="s">
-        <v>22</v>
-      </c>
-      <c r="G50" t="s">
-        <v>22</v>
-      </c>
-      <c r="H50" t="s">
-        <v>22</v>
-      </c>
-      <c r="I50" t="s">
-        <v>22</v>
-      </c>
-      <c r="J50" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" t="s">
-        <v>21</v>
-      </c>
-      <c r="E51" t="s">
-        <v>16</v>
-      </c>
-      <c r="F51" t="s">
-        <v>22</v>
-      </c>
-      <c r="G51" t="s">
-        <v>22</v>
-      </c>
-      <c r="H51" t="s">
-        <v>22</v>
-      </c>
-      <c r="I51" t="s">
-        <v>22</v>
-      </c>
-      <c r="J51" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10">
-      <c r="A52" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H52" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I52" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J52" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10">
-      <c r="A54" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I54" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J54" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D55" t="s">
         <v>20</v>
@@ -3728,24 +3825,24 @@
         <v>16</v>
       </c>
       <c r="F55" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="G55" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H55" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I55" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>46</v>
+        <v>118</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B56" t="s">
         <v>13</v>
@@ -3774,7 +3871,7 @@
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>14</v>
@@ -3804,10 +3901,10 @@
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="1" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2" t="s">
@@ -3834,25 +3931,25 @@
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B60" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D60" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E60" t="s">
         <v>16</v>
       </c>
       <c r="F60" t="s">
-        <v>111</v>
+        <v>63</v>
       </c>
       <c r="G60" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="H60" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="I60" t="s">
         <v>16</v>
@@ -3863,118 +3960,91 @@
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" t="s">
+        <v>21</v>
+      </c>
+      <c r="E61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>22</v>
+      </c>
+      <c r="G61" t="s">
+        <v>22</v>
+      </c>
+      <c r="H61" t="s">
+        <v>22</v>
+      </c>
+      <c r="I61" t="s">
+        <v>22</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I62" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J62" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B61" t="s">
-        <v>120</v>
-      </c>
-      <c r="D61" t="s">
-        <v>45</v>
-      </c>
-      <c r="E61" t="s">
-        <v>16</v>
-      </c>
-      <c r="F61" t="s">
-        <v>24</v>
-      </c>
-      <c r="G61" t="s">
-        <v>72</v>
-      </c>
-      <c r="H61" t="s">
-        <v>45</v>
-      </c>
-      <c r="I61" t="s">
-        <v>16</v>
-      </c>
-      <c r="J61" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10">
-      <c r="A62" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B62" t="s">
-        <v>133</v>
-      </c>
-      <c r="D62" t="s">
-        <v>45</v>
-      </c>
-      <c r="E62" t="s">
-        <v>16</v>
-      </c>
-      <c r="F62" t="s">
-        <v>126</v>
-      </c>
-      <c r="G62" t="s">
-        <v>127</v>
-      </c>
-      <c r="H62" t="s">
-        <v>45</v>
-      </c>
-      <c r="I62" t="s">
-        <v>16</v>
-      </c>
-      <c r="J62" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10">
-      <c r="A63" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B63" t="s">
-        <v>10</v>
-      </c>
-      <c r="D63" t="s">
-        <v>45</v>
-      </c>
-      <c r="E63" t="s">
-        <v>16</v>
-      </c>
-      <c r="F63" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G63" t="s">
-        <v>10</v>
-      </c>
-      <c r="H63" t="s">
-        <v>45</v>
-      </c>
-      <c r="I63" t="s">
-        <v>16</v>
-      </c>
-      <c r="J63" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10">
-      <c r="A64" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B64" t="s">
-        <v>66</v>
-      </c>
-      <c r="D64" t="s">
-        <v>20</v>
-      </c>
-      <c r="E64" t="s">
-        <v>16</v>
-      </c>
-      <c r="F64" t="s">
-        <v>111</v>
-      </c>
-      <c r="G64" t="s">
-        <v>66</v>
-      </c>
-      <c r="H64" t="s">
-        <v>20</v>
-      </c>
-      <c r="I64" t="s">
-        <v>16</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>46</v>
+      <c r="B64" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -3982,10 +4052,10 @@
         <v>49</v>
       </c>
       <c r="B65" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D65" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E65" t="s">
         <v>16</v>
@@ -3994,16 +4064,16 @@
         <v>111</v>
       </c>
       <c r="G65" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H65" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I65" t="s">
         <v>16</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>123</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -4011,122 +4081,149 @@
         <v>49</v>
       </c>
       <c r="B66" t="s">
-        <v>13</v>
+        <v>120</v>
       </c>
       <c r="D66" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="E66" t="s">
         <v>16</v>
       </c>
       <c r="F66" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G66" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="H66" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="I66" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>18</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" spans="1:10">
-      <c r="A67" s="6" t="s">
+      <c r="A67" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B67" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F67" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G67" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I67" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J67" s="8" t="s">
-        <v>19</v>
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+      <c r="D67" t="s">
+        <v>45</v>
+      </c>
+      <c r="E67" t="s">
+        <v>16</v>
+      </c>
+      <c r="F67" t="s">
+        <v>126</v>
+      </c>
+      <c r="G67" t="s">
+        <v>127</v>
+      </c>
+      <c r="H67" t="s">
+        <v>45</v>
+      </c>
+      <c r="I67" t="s">
+        <v>16</v>
+      </c>
+      <c r="J67" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B68" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" t="s">
+        <v>45</v>
+      </c>
+      <c r="E68" t="s">
+        <v>16</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G68" t="s">
+        <v>10</v>
+      </c>
+      <c r="H68" t="s">
+        <v>45</v>
+      </c>
+      <c r="I68" t="s">
+        <v>16</v>
+      </c>
+      <c r="J68" s="5" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:10">
-      <c r="A69" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H69" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I69" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J69" s="3" t="s">
-        <v>130</v>
+      <c r="A69" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B69" t="s">
+        <v>66</v>
+      </c>
+      <c r="D69" t="s">
+        <v>20</v>
+      </c>
+      <c r="E69" t="s">
+        <v>16</v>
+      </c>
+      <c r="F69" t="s">
+        <v>111</v>
+      </c>
+      <c r="G69" t="s">
+        <v>66</v>
+      </c>
+      <c r="H69" t="s">
+        <v>20</v>
+      </c>
+      <c r="I69" t="s">
+        <v>16</v>
+      </c>
+      <c r="J69" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
       <c r="B70" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D70" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E70" t="s">
         <v>16</v>
       </c>
       <c r="F70" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
       <c r="G70" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H70" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="I70" t="s">
         <v>16</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
       <c r="B71" t="s">
         <v>13</v>
@@ -4155,7 +4252,7 @@
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="6" t="s">
-        <v>129</v>
+        <v>49</v>
       </c>
       <c r="B72" s="7" t="s">
         <v>14</v>
@@ -4180,6 +4277,124 @@
         <v>22</v>
       </c>
       <c r="J72" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10">
+      <c r="A74" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C74" s="2"/>
+      <c r="D74" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10">
+      <c r="A75" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B75" t="s">
+        <v>60</v>
+      </c>
+      <c r="D75" t="s">
+        <v>45</v>
+      </c>
+      <c r="E75" t="s">
+        <v>16</v>
+      </c>
+      <c r="F75" t="s">
+        <v>48</v>
+      </c>
+      <c r="G75" t="s">
+        <v>60</v>
+      </c>
+      <c r="H75" t="s">
+        <v>45</v>
+      </c>
+      <c r="I75" t="s">
+        <v>16</v>
+      </c>
+      <c r="J75" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10">
+      <c r="A76" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B76" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" t="s">
+        <v>21</v>
+      </c>
+      <c r="E76" t="s">
+        <v>16</v>
+      </c>
+      <c r="F76" t="s">
+        <v>22</v>
+      </c>
+      <c r="G76" t="s">
+        <v>22</v>
+      </c>
+      <c r="H76" t="s">
+        <v>22</v>
+      </c>
+      <c r="I76" t="s">
+        <v>22</v>
+      </c>
+      <c r="J76" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10">
+      <c r="A77" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F77" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I77" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J77" s="8" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>